<commit_message>
Fix Excel workbook compatibility
</commit_message>
<xml_diff>
--- a/examples/Expected_Workbook_Format.xlsx
+++ b/examples/Expected_Workbook_Format.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sentences" sheetId="1" r:id="R27001edbbb3f4020"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="2" r:id="Rce7a987108e948b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sentences" sheetId="1" r:id="Ra56c576cd98d4e3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="2" r:id="Rd9ac17bc96d24967"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -134,43 +134,6 @@
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SentencesTable" displayName="SentencesTable" ref="A1:D3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="4">
-    <x:tableColumn id="1" name="Foreign-language verb"/>
-    <x:tableColumn id="2" name="Verb translation"/>
-    <x:tableColumn id="3" name="Foreign-language sentence"/>
-    <x:tableColumn id="4" name="Sentence translation"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MetadataTable" displayName="MetadataTable" ref="A1:Q3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="17">
-    <x:tableColumn id="1" name="Row number"/>
-    <x:tableColumn id="2" name="Base item"/>
-    <x:tableColumn id="3" name="CEFR level"/>
-    <x:tableColumn id="4" name="Frequency rank"/>
-    <x:tableColumn id="5" name="Grammatical person"/>
-    <x:tableColumn id="6" name="Tense/form"/>
-    <x:tableColumn id="7" name="Question/statement"/>
-    <x:tableColumn id="8" name="Generation timestamp"/>
-    <x:tableColumn id="9" name="Provider"/>
-    <x:tableColumn id="10" name="Model"/>
-    <x:tableColumn id="11" name="Validation status"/>
-    <x:tableColumn id="12" name="Random seed"/>
-    <x:tableColumn id="13" name="Input tokens"/>
-    <x:tableColumn id="14" name="Output tokens"/>
-    <x:tableColumn id="15" name="Estimated cost USD"/>
-    <x:tableColumn id="16" name="Actual cost USD"/>
-    <x:tableColumn id="17" name="Generation settings"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -418,9 +381,6 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b564347f93549f4"/>
-  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -608,8 +568,5 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fbdb04abb3f4f9c"/>
-  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: expand generation to 5000 ranked words
</commit_message>
<xml_diff>
--- a/examples/Expected_Workbook_Format.xlsx
+++ b/examples/Expected_Workbook_Format.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sentences" sheetId="1" r:id="Ra56c576cd98d4e3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="2" r:id="Rd9ac17bc96d24967"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sentences" sheetId="1" r:id="R2c0a523dee494c37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="2" r:id="R5e2700d1d2fa4058"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +15,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="1">
-    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd hh:mm:ss"/>
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd hh:mm"/>
   </x:numFmts>
   <x:fonts count="3">
     <x:font>
@@ -23,18 +23,18 @@
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF172033"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF172033"/>
-      <x:name val="Carlito"/>
+      <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -46,89 +46,190 @@
         <x:fgColor rgb="FF2E74B5"/>
       </x:patternFill>
     </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFF7F9FC"/>
-      </x:patternFill>
-    </x:fill>
   </x:fills>
-  <x:borders count="7">
+  <x:borders count="10">
     <x:border/>
     <x:border>
       <x:right style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:right>
       <x:bottom style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:left>
       <x:right style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:right>
       <x:bottom style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:left>
       <x:bottom style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:right style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD8E0EA"/>
       </x:top>
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:left>
       <x:right style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:top>
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:left>
       <x:top style="thin">
-        <x:color rgb="FFD7E0EA"/>
+        <x:color rgb="FFD8E0EA"/>
       </x:top>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="36">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -333,50 +434,78 @@
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="24" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Foreign-language verb</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="str">
-        <x:v>Verb translation</x:v>
-      </x:c>
-      <x:c r="C1" s="3" t="str">
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="32" t="str">
+        <x:v>Foreign-language word</x:v>
+      </x:c>
+      <x:c r="B1" s="33" t="str">
+        <x:v>Word translation</x:v>
+      </x:c>
+      <x:c r="C1" s="33" t="str">
         <x:v>Foreign-language sentence</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="str">
+      <x:c r="D1" s="34" t="str">
         <x:v>Sentence translation</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="6" t="str">
-        <x:v>lernen</x:v>
-      </x:c>
-      <x:c r="B2" s="7" t="str">
-        <x:v>to learn</x:v>
-      </x:c>
-      <x:c r="C2" s="7" t="str">
-        <x:v>Ich lerne jeden Tag.</x:v>
-      </x:c>
-      <x:c r="D2" s="8" t="str">
-        <x:v>I learn every day.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="9" t="str">
-        <x:v>fragen</x:v>
-      </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>to ask</x:v>
-      </x:c>
-      <x:c r="C3" s="10" t="str">
-        <x:v>Fragst du den Lehrer?</x:v>
-      </x:c>
-      <x:c r="D3" s="11" t="str">
-        <x:v>Are you asking the teacher?</x:v>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="23" t="str">
+        <x:v>sein</x:v>
+      </x:c>
+      <x:c r="B2" s="24" t="str">
+        <x:v>to be</x:v>
+      </x:c>
+      <x:c r="C2" s="24" t="str">
+        <x:v>Ich bin heute hier.</x:v>
+      </x:c>
+      <x:c r="D2" s="25" t="str">
+        <x:v>I am here today.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="23" t="str">
+        <x:v>Werkzeug</x:v>
+      </x:c>
+      <x:c r="B3" s="24" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="C3" s="24" t="str">
+        <x:v>Das Werkzeug liegt dort.</x:v>
+      </x:c>
+      <x:c r="D3" s="25" t="str">
+        <x:v>The tool is lying there.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="23" t="str">
+        <x:v>gut</x:v>
+      </x:c>
+      <x:c r="B4" s="24" t="str">
+        <x:v>good</x:v>
+      </x:c>
+      <x:c r="C4" s="24" t="str">
+        <x:v>Das ist eine gute Idee.</x:v>
+      </x:c>
+      <x:c r="D4" s="25" t="str">
+        <x:v>That is a good idea.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="26" t="str">
+        <x:v>immer</x:v>
+      </x:c>
+      <x:c r="B5" s="27" t="str">
+        <x:v>always</x:v>
+      </x:c>
+      <x:c r="C5" s="27" t="str">
+        <x:v>Kommst du immer pünktlich?</x:v>
+      </x:c>
+      <x:c r="D5" s="28" t="str">
+        <x:v>Do you always arrive on time?</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -388,181 +517,303 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="8.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="9" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16.219999313354492" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="15.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="7.110000133514404" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="13.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="11.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="10.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="11.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="13.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="32" t="str">
         <x:v>Row number</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="str">
+      <x:c r="B1" s="33" t="str">
         <x:v>Base item</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="str">
+      <x:c r="C1" s="33" t="str">
         <x:v>CEFR level</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="str">
+      <x:c r="D1" s="33" t="str">
         <x:v>Frequency rank</x:v>
       </x:c>
-      <x:c r="E1" s="3" t="str">
+      <x:c r="E1" s="33" t="str">
+        <x:v>Part of speech</x:v>
+      </x:c>
+      <x:c r="F1" s="33" t="str">
         <x:v>Grammatical person</x:v>
       </x:c>
-      <x:c r="F1" s="3" t="str">
-        <x:v>Tense/form</x:v>
-      </x:c>
-      <x:c r="G1" s="3" t="str">
+      <x:c r="G1" s="33" t="str">
+        <x:v>Word form/variant</x:v>
+      </x:c>
+      <x:c r="H1" s="33" t="str">
         <x:v>Question/statement</x:v>
       </x:c>
-      <x:c r="H1" s="3" t="str">
+      <x:c r="I1" s="35" t="str">
         <x:v>Generation timestamp</x:v>
       </x:c>
-      <x:c r="I1" s="3" t="str">
+      <x:c r="J1" s="33" t="str">
         <x:v>Provider</x:v>
       </x:c>
-      <x:c r="J1" s="3" t="str">
+      <x:c r="K1" s="33" t="str">
         <x:v>Model</x:v>
       </x:c>
-      <x:c r="K1" s="3" t="str">
+      <x:c r="L1" s="33" t="str">
         <x:v>Validation status</x:v>
       </x:c>
-      <x:c r="L1" s="3" t="str">
+      <x:c r="M1" s="33" t="str">
         <x:v>Random seed</x:v>
       </x:c>
-      <x:c r="M1" s="3" t="str">
+      <x:c r="N1" s="33" t="str">
         <x:v>Input tokens</x:v>
       </x:c>
-      <x:c r="N1" s="3" t="str">
+      <x:c r="O1" s="33" t="str">
         <x:v>Output tokens</x:v>
       </x:c>
-      <x:c r="O1" s="3" t="str">
+      <x:c r="P1" s="33" t="str">
         <x:v>Estimated cost USD</x:v>
       </x:c>
-      <x:c r="P1" s="3" t="str">
+      <x:c r="Q1" s="33" t="str">
         <x:v>Actual cost USD</x:v>
       </x:c>
-      <x:c r="Q1" s="3" t="str">
+      <x:c r="R1" s="34" t="str">
         <x:v>Generation settings</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="6" t="n">
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="23" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B2" s="7" t="n">
+      <x:c r="B2" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C2" s="7" t="str">
+      <x:c r="C2" s="24" t="str">
         <x:v>A1</x:v>
       </x:c>
-      <x:c r="D2" s="7" t="n">
+      <x:c r="D2" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E2" s="7" t="str">
+      <x:c r="E2" s="24" t="str">
+        <x:v>verb</x:v>
+      </x:c>
+      <x:c r="F2" s="24" t="str">
         <x:v>first_singular</x:v>
       </x:c>
-      <x:c r="F2" s="7" t="str">
+      <x:c r="G2" s="24" t="str">
         <x:v>present</x:v>
       </x:c>
-      <x:c r="G2" s="7" t="str">
+      <x:c r="H2" s="24" t="str">
         <x:v>statement</x:v>
       </x:c>
-      <x:c r="H2" s="12" t="n">
-        <x:v>46254.5</x:v>
-      </x:c>
-      <x:c r="I2" s="7" t="str">
+      <x:c r="I2" s="24" t="n">
+        <x:v>46258.5</x:v>
+      </x:c>
+      <x:c r="J2" s="24" t="str">
         <x:v>Example</x:v>
       </x:c>
-      <x:c r="J2" s="7" t="str">
+      <x:c r="K2" s="24" t="str">
         <x:v>Example model</x:v>
       </x:c>
-      <x:c r="K2" s="7" t="str">
+      <x:c r="L2" s="24" t="str">
         <x:v>accepted</x:v>
       </x:c>
-      <x:c r="L2" s="7" t="n">
+      <x:c r="M2" s="24" t="n">
         <x:v>12345</x:v>
       </x:c>
-      <x:c r="M2" s="7" t="n">
+      <x:c r="N2" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N2" s="7" t="n">
+      <x:c r="O2" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O2" s="7" t="str">
+      <x:c r="P2" s="24" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="P2" s="7" t="str">
+      <x:c r="Q2" s="24" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="Q2" s="8" t="str">
+      <x:c r="R2" s="25" t="str">
         <x:v>Example settings</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="9" t="n">
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="23" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="n">
+      <x:c r="B3" s="24" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C3" s="10" t="str">
+      <x:c r="C3" s="24" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="D3" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E3" s="24" t="str">
+        <x:v>noun</x:v>
+      </x:c>
+      <x:c r="F3" s="24" t="str">
+        <x:v>third_singular</x:v>
+      </x:c>
+      <x:c r="G3" s="24" t="str">
+        <x:v>singular</x:v>
+      </x:c>
+      <x:c r="H3" s="24" t="str">
+        <x:v>statement</x:v>
+      </x:c>
+      <x:c r="I3" s="24" t="n">
+        <x:v>46258.5</x:v>
+      </x:c>
+      <x:c r="J3" s="24" t="str">
+        <x:v>Example</x:v>
+      </x:c>
+      <x:c r="K3" s="24" t="str">
+        <x:v>Example model</x:v>
+      </x:c>
+      <x:c r="L3" s="24" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="M3" s="24" t="n">
+        <x:v>12345</x:v>
+      </x:c>
+      <x:c r="N3" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O3" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P3" s="24" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="Q3" s="24" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="R3" s="25" t="str">
+        <x:v>Example settings</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="24" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C4" s="24" t="str">
         <x:v>A2</x:v>
       </x:c>
-      <x:c r="D3" s="10" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E3" s="10" t="str">
+      <x:c r="D4" s="24" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E4" s="24" t="str">
+        <x:v>adjective</x:v>
+      </x:c>
+      <x:c r="F4" s="24" t="str">
+        <x:v>third_singular</x:v>
+      </x:c>
+      <x:c r="G4" s="24" t="str">
+        <x:v>feminine nominative</x:v>
+      </x:c>
+      <x:c r="H4" s="24" t="str">
+        <x:v>statement</x:v>
+      </x:c>
+      <x:c r="I4" s="24" t="n">
+        <x:v>46258.5</x:v>
+      </x:c>
+      <x:c r="J4" s="24" t="str">
+        <x:v>Example</x:v>
+      </x:c>
+      <x:c r="K4" s="24" t="str">
+        <x:v>Example model</x:v>
+      </x:c>
+      <x:c r="L4" s="24" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="M4" s="24" t="n">
+        <x:v>12345</x:v>
+      </x:c>
+      <x:c r="N4" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O4" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P4" s="24" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="Q4" s="24" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="R4" s="25" t="str">
+        <x:v>Example settings</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="26" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="27" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="27" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D5" s="27" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E5" s="27" t="str">
+        <x:v>adverb</x:v>
+      </x:c>
+      <x:c r="F5" s="27" t="str">
         <x:v>second_singular</x:v>
       </x:c>
-      <x:c r="F3" s="10" t="str">
-        <x:v>present</x:v>
-      </x:c>
-      <x:c r="G3" s="10" t="str">
+      <x:c r="G5" s="27" t="str">
+        <x:v>invariant-context-1</x:v>
+      </x:c>
+      <x:c r="H5" s="27" t="str">
         <x:v>question</x:v>
       </x:c>
-      <x:c r="H3" s="13" t="n">
-        <x:v>46254.5</x:v>
-      </x:c>
-      <x:c r="I3" s="10" t="str">
+      <x:c r="I5" s="27" t="n">
+        <x:v>46258.5</x:v>
+      </x:c>
+      <x:c r="J5" s="27" t="str">
         <x:v>Example</x:v>
       </x:c>
-      <x:c r="J3" s="10" t="str">
+      <x:c r="K5" s="27" t="str">
         <x:v>Example model</x:v>
       </x:c>
-      <x:c r="K3" s="10" t="str">
+      <x:c r="L5" s="27" t="str">
         <x:v>accepted</x:v>
       </x:c>
-      <x:c r="L3" s="10" t="n">
+      <x:c r="M5" s="27" t="n">
         <x:v>12345</x:v>
       </x:c>
-      <x:c r="M3" s="10" t="n">
+      <x:c r="N5" s="27" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N3" s="10" t="n">
+      <x:c r="O5" s="27" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O3" s="10" t="str">
+      <x:c r="P5" s="27" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="P3" s="10" t="str">
+      <x:c r="Q5" s="27" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="Q3" s="11" t="str">
+      <x:c r="R5" s="28" t="str">
         <x:v>Example settings</x:v>
       </x:c>
     </x:row>

</xml_diff>